<commit_message>
Corrige sync Mogo sem substituir arquivos conferidos
- trava replace por padrão no organizar_drive_mogo.py\n- adiciona auditoria dos 77 arquivos substituídos no Drive\n- salva backfill histórico e relatórios Mogo gerados
</commit_message>
<xml_diff>
--- a/relatorios/Mogo/Analise Quantidades Produzidas/03-2026.xlsx
+++ b/relatorios/Mogo/Analise Quantidades Produzidas/03-2026.xlsx
@@ -57,11 +57,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -487,15 +488,11 @@
           <t>5,000</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>5,91</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>29,57</t>
-        </is>
+      <c r="C2" s="2" t="n">
+        <v>5.91</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>29.57</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -524,15 +521,11 @@
           <t>8,100</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>20,50</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>166,02</t>
-        </is>
+      <c r="C3" s="2" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>166.02</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -561,15 +554,11 @@
           <t>6,000</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>11,98</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>71,85</t>
-        </is>
+      <c r="C4" s="2" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>71.84999999999999</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -598,15 +587,11 @@
           <t>10,000</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>5,99</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>59,88</t>
-        </is>
+      <c r="C5" s="2" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>59.88</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -635,15 +620,11 @@
           <t>13,000</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2,99</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>38,92</t>
-        </is>
+      <c r="C6" s="2" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>38.92</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -672,15 +653,11 @@
           <t>16,800</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>9,98</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>167,66</t>
-        </is>
+      <c r="C7" s="2" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>167.66</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -709,15 +686,11 @@
           <t>91,000</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>7,49</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>681,83</t>
-        </is>
+      <c r="C8" s="2" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>681.83</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -746,15 +719,11 @@
           <t>66,000</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1,75</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>115,60</t>
-        </is>
+      <c r="C9" s="2" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>115.6</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -783,15 +752,11 @@
           <t>43,000</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>3,47</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>149,34</t>
-        </is>
+      <c r="C10" s="2" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>149.34</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -820,15 +785,11 @@
           <t>133,000</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>5,35</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>711,34</t>
-        </is>
+      <c r="C11" s="2" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>711.34</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -857,15 +818,11 @@
           <t>72,000</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1,39</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>100,02</t>
-        </is>
+      <c r="C12" s="2" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>100.02</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -894,15 +851,11 @@
           <t>5,220</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>7,28</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>38,00</t>
-        </is>
+      <c r="C13" s="2" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>38</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -931,15 +884,11 @@
           <t>140,140</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>6,95</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>973,42</t>
-        </is>
+      <c r="C14" s="2" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>973.42</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -968,15 +917,11 @@
           <t>9,540</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>7,65</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>72,97</t>
-        </is>
+      <c r="C15" s="2" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>72.97</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1005,15 +950,11 @@
           <t>153,140</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>9,73</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>1.490,17</t>
-        </is>
+      <c r="C16" s="2" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>1490.17</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1042,15 +983,11 @@
           <t>6,000</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>32,65</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>195,92</t>
-        </is>
+      <c r="C17" s="2" t="n">
+        <v>32.65</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>195.92</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1079,15 +1016,11 @@
           <t>11,000</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>19,37</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>213,12</t>
-        </is>
+      <c r="C18" s="2" t="n">
+        <v>19.37</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>213.12</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1116,15 +1049,11 @@
           <t>6,000</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>22,36</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>134,17</t>
-        </is>
+      <c r="C19" s="2" t="n">
+        <v>22.36</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>134.17</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1153,15 +1082,11 @@
           <t>11,000</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>12,45</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>136,90</t>
-        </is>
+      <c r="C20" s="2" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>136.9</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1190,15 +1115,11 @@
           <t>6,000</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>7,02</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>42,13</t>
-        </is>
+      <c r="C21" s="2" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>42.13</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1227,15 +1148,11 @@
           <t>11,000</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>3,95</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>43,45</t>
-        </is>
+      <c r="C22" s="2" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>43.45</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1264,15 +1181,11 @@
           <t>4,600</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>21,94</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>100,94</t>
-        </is>
+      <c r="C23" s="2" t="n">
+        <v>21.94</v>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>100.94</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1301,15 +1214,11 @@
           <t>10,000</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>45,94</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>459,35</t>
-        </is>
+      <c r="C24" s="2" t="n">
+        <v>45.94</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>459.35</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1338,15 +1247,11 @@
           <t>10,000</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>37,36</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>373,57</t>
-        </is>
+      <c r="C25" s="2" t="n">
+        <v>37.36</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>373.57</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1375,15 +1280,11 @@
           <t>10,730</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>29,76</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>319,28</t>
-        </is>
+      <c r="C26" s="2" t="n">
+        <v>29.76</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>319.28</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1412,15 +1313,11 @@
           <t>9,000</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>13,41</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>120,73</t>
-        </is>
+      <c r="C27" s="2" t="n">
+        <v>13.41</v>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>120.73</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1449,15 +1346,11 @@
           <t>24,000</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>2,19</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>52,51</t>
-        </is>
+      <c r="C28" s="2" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>52.51</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1486,15 +1379,11 @@
           <t>8,000</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>10,94</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>87,51</t>
-        </is>
+      <c r="C29" s="2" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>87.51000000000001</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1523,15 +1412,11 @@
           <t>8,000</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>10,94</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>87,51</t>
-        </is>
+      <c r="C30" s="2" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>87.51000000000001</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1560,15 +1445,11 @@
           <t>24,000</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>2,19</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>52,51</t>
-        </is>
+      <c r="C31" s="2" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>52.51</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1597,15 +1478,11 @@
           <t>10,000</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>7,28</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>72,80</t>
-        </is>
+      <c r="C32" s="2" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>72.8</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1634,15 +1511,11 @@
           <t>6,000</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>3,92</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>23,51</t>
-        </is>
+      <c r="C33" s="2" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>23.51</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1671,15 +1544,11 @@
           <t>13,440</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>22,89</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>307,66</t>
-        </is>
+      <c r="C34" s="2" t="n">
+        <v>22.89</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>307.66</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1708,15 +1577,11 @@
           <t>13,000</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>30,00</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>390,01</t>
-        </is>
+      <c r="C35" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>390.01</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1745,15 +1610,11 @@
           <t>6,400</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>13,75</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>87,98</t>
-        </is>
+      <c r="C36" s="2" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>87.98</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1782,15 +1643,11 @@
           <t>19,540</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>21,88</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>427,48</t>
-        </is>
+      <c r="C37" s="2" t="n">
+        <v>21.88</v>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>427.48</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1819,15 +1676,11 @@
           <t>4,000</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>27,05</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>108,20</t>
-        </is>
+      <c r="C38" s="2" t="n">
+        <v>27.05</v>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>108.2</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1856,15 +1709,11 @@
           <t>12,000</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>14,95</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>179,40</t>
-        </is>
+      <c r="C39" s="2" t="n">
+        <v>14.95</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>179.4</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1893,15 +1742,11 @@
           <t>8,000</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>39,65</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>317,20</t>
-        </is>
+      <c r="C40" s="2" t="n">
+        <v>39.65</v>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>317.2</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1930,15 +1775,11 @@
           <t>7,360</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>7,47</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>54,99</t>
-        </is>
+      <c r="C41" s="2" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>54.99</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1967,15 +1808,11 @@
           <t>9,700</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>16,04</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>155,54</t>
-        </is>
+      <c r="C42" s="2" t="n">
+        <v>16.04</v>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>155.54</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2004,15 +1841,11 @@
           <t>12,320</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>22,90</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>282,11</t>
-        </is>
+      <c r="C43" s="2" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>282.11</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2041,15 +1874,11 @@
           <t>8,000</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>7,29</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>58,33</t>
-        </is>
+      <c r="C44" s="2" t="n">
+        <v>7.29</v>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>58.33</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -2078,15 +1907,11 @@
           <t>12,000</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>2,43</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>29,17</t>
-        </is>
+      <c r="C45" s="2" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>29.17</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2115,15 +1940,11 @@
           <t>3,410</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>23,33</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>79,56</t>
-        </is>
+      <c r="C46" s="2" t="n">
+        <v>23.33</v>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>79.56</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -2152,15 +1973,11 @@
           <t>6,000</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>13,30</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>79,80</t>
-        </is>
+      <c r="C47" s="2" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>79.8</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2189,15 +2006,11 @@
           <t>9,700</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>16,04</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>155,54</t>
-        </is>
+      <c r="C48" s="2" t="n">
+        <v>16.04</v>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>155.54</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -2226,15 +2039,11 @@
           <t>66,000</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>5,28</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>348,46</t>
-        </is>
+      <c r="C49" s="2" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>348.46</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -2263,15 +2072,11 @@
           <t>4,560</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>21,35</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>97,34</t>
-        </is>
+      <c r="C50" s="2" t="n">
+        <v>21.35</v>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>97.34</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -2300,15 +2105,11 @@
           <t>19,540</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>21,88</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>427,48</t>
-        </is>
+      <c r="C51" s="2" t="n">
+        <v>21.88</v>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>427.48</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -2337,15 +2138,11 @@
           <t>5,200</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>27,52</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>143,10</t>
-        </is>
+      <c r="C52" s="2" t="n">
+        <v>27.52</v>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>143.1</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -2374,15 +2171,11 @@
           <t>6,000</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>15,17</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>91,01</t>
-        </is>
+      <c r="C53" s="2" t="n">
+        <v>15.17</v>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>91.01000000000001</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -2411,15 +2204,11 @@
           <t>5,220</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>7,28</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>38,00</t>
-        </is>
+      <c r="C54" s="2" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>38</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -2448,15 +2237,11 @@
           <t>45,600</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>20,04</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>913,80</t>
-        </is>
+      <c r="C55" s="2" t="n">
+        <v>20.04</v>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>913.8</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -2485,15 +2270,11 @@
           <t>12,000</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>3,48</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>41,77</t>
-        </is>
+      <c r="C56" s="2" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>41.77</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -2522,15 +2303,11 @@
           <t>11,000</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>15,49</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>170,39</t>
-        </is>
+      <c r="C57" s="2" t="n">
+        <v>15.49</v>
+      </c>
+      <c r="D57" s="2" t="n">
+        <v>170.39</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2559,15 +2336,11 @@
           <t>12,000</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>6,40</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>76,81</t>
-        </is>
+      <c r="C58" s="2" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>76.81</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -2596,15 +2369,11 @@
           <t>15,000</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>14,95</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>224,25</t>
-        </is>
+      <c r="C59" s="2" t="n">
+        <v>14.95</v>
+      </c>
+      <c r="D59" s="2" t="n">
+        <v>224.25</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -2633,15 +2402,11 @@
           <t>4,000</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>13,30</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>53,20</t>
-        </is>
+      <c r="C60" s="2" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>53.2</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2670,15 +2435,11 @@
           <t>9,000</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>30,00</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>270,00</t>
-        </is>
+      <c r="C61" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D61" s="2" t="n">
+        <v>270</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -2707,15 +2468,11 @@
           <t>15,000</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>2,43</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>36,44</t>
-        </is>
+      <c r="C62" s="2" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>36.44</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -2744,15 +2501,11 @@
           <t>7,500</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>10,86</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>81,46</t>
-        </is>
+      <c r="C63" s="2" t="n">
+        <v>10.86</v>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>81.45999999999999</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -2781,15 +2534,11 @@
           <t>9,540</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>7,65</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>72,97</t>
-        </is>
+      <c r="C64" s="2" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>72.97</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2818,15 +2567,11 @@
           <t>1,550</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>23,36</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>36,21</t>
-        </is>
+      <c r="C65" s="2" t="n">
+        <v>23.36</v>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>36.21</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2855,15 +2600,11 @@
           <t>9,700</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>16,04</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>155,54</t>
-        </is>
+      <c r="C66" s="2" t="n">
+        <v>16.04</v>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>155.54</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2892,15 +2633,11 @@
           <t>6,400</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>13,75</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>87,98</t>
-        </is>
+      <c r="C67" s="2" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>87.98</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2929,15 +2666,11 @@
           <t>11,000</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>11,98</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>131,73</t>
-        </is>
+      <c r="C68" s="2" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>131.73</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2966,15 +2699,11 @@
           <t>10,000</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>5,99</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>59,88</t>
-        </is>
+      <c r="C69" s="2" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>59.88</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -3003,15 +2732,11 @@
           <t>9,700</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>16,04</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>155,54</t>
-        </is>
+      <c r="C70" s="2" t="n">
+        <v>16.04</v>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>155.54</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -3040,15 +2765,11 @@
           <t>6,240</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>15,47</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>96,55</t>
-        </is>
+      <c r="C71" s="2" t="n">
+        <v>15.47</v>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>96.55</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -3077,15 +2798,11 @@
           <t>19,200</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>9,98</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>191,61</t>
-        </is>
+      <c r="C72" s="2" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>191.61</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -3114,15 +2831,11 @@
           <t>4,770</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>7,65</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>36,49</t>
-        </is>
+      <c r="C73" s="2" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>36.49</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -3151,15 +2864,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>4,27</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>4,27</t>
-        </is>
+      <c r="C74" s="2" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>4.27</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -3188,15 +2897,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>8,95</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>8,95</t>
-        </is>
+      <c r="C75" s="2" t="n">
+        <v>8.949999999999999</v>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>8.949999999999999</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3225,15 +2930,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>11,02</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>11,02</t>
-        </is>
+      <c r="C76" s="2" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>11.02</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -3262,15 +2963,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>3,95</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>3,95</t>
-        </is>
+      <c r="C77" s="2" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>3.95</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -3299,15 +2996,11 @@
           <t>9,930</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>15,33</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>152,25</t>
-        </is>
+      <c r="C78" s="2" t="n">
+        <v>15.33</v>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>152.25</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -3336,15 +3029,11 @@
           <t>7,100</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>17,87</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>126,88</t>
-        </is>
+      <c r="C79" s="2" t="n">
+        <v>17.87</v>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>126.88</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -3373,15 +3062,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>6,32</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>6,32</t>
-        </is>
+      <c r="C80" s="2" t="n">
+        <v>6.32</v>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>6.32</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -3410,15 +3095,11 @@
           <t>4,000</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>3,35</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>13,41</t>
-        </is>
+      <c r="C81" s="2" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>13.41</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -3447,15 +3128,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>9,54</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>9,54</t>
-        </is>
+      <c r="C82" s="2" t="n">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>9.539999999999999</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -3484,15 +3161,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>6,37</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>6,37</t>
-        </is>
+      <c r="C83" s="2" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>6.37</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -3521,15 +3194,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>9,15</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>9,15</t>
-        </is>
+      <c r="C84" s="2" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>9.15</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -3558,15 +3227,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>9,54</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>9,54</t>
-        </is>
+      <c r="C85" s="2" t="n">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="D85" s="2" t="n">
+        <v>9.539999999999999</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -3595,15 +3260,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>15,08</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>15,08</t>
-        </is>
+      <c r="C86" s="2" t="n">
+        <v>15.08</v>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>15.08</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -3632,15 +3293,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>7,21</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>7,21</t>
-        </is>
+      <c r="C87" s="2" t="n">
+        <v>7.21</v>
+      </c>
+      <c r="D87" s="2" t="n">
+        <v>7.21</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -3669,15 +3326,11 @@
           <t>4,000</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>6,41</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>25,62</t>
-        </is>
+      <c r="C88" s="2" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="D88" s="2" t="n">
+        <v>25.62</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -3706,15 +3359,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>9,97</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>9,97</t>
-        </is>
+      <c r="C89" s="2" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="D89" s="2" t="n">
+        <v>9.970000000000001</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -3743,15 +3392,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>11,28</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>11,28</t>
-        </is>
+      <c r="C90" s="2" t="n">
+        <v>11.28</v>
+      </c>
+      <c r="D90" s="2" t="n">
+        <v>11.28</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -3780,15 +3425,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>7,20</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>7,20</t>
-        </is>
+      <c r="C91" s="2" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="D91" s="2" t="n">
+        <v>7.2</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -3817,15 +3458,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>6,43</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>6,43</t>
-        </is>
+      <c r="C92" s="2" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="D92" s="2" t="n">
+        <v>6.43</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -3854,15 +3491,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>48,08</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>48,08</t>
-        </is>
+      <c r="C93" s="2" t="n">
+        <v>48.08</v>
+      </c>
+      <c r="D93" s="2" t="n">
+        <v>48.08</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -3891,15 +3524,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>22,85</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>22,85</t>
-        </is>
+      <c r="C94" s="2" t="n">
+        <v>22.85</v>
+      </c>
+      <c r="D94" s="2" t="n">
+        <v>22.85</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -3928,15 +3557,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>19,39</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>19,39</t>
-        </is>
+      <c r="C95" s="2" t="n">
+        <v>19.39</v>
+      </c>
+      <c r="D95" s="2" t="n">
+        <v>19.39</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -3965,15 +3590,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>14,62</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>14,62</t>
-        </is>
+      <c r="C96" s="2" t="n">
+        <v>14.62</v>
+      </c>
+      <c r="D96" s="2" t="n">
+        <v>14.62</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -4002,15 +3623,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>14,69</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>14,69</t>
-        </is>
+      <c r="C97" s="2" t="n">
+        <v>14.69</v>
+      </c>
+      <c r="D97" s="2" t="n">
+        <v>14.69</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -4039,15 +3656,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>21,23</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>21,23</t>
-        </is>
+      <c r="C98" s="2" t="n">
+        <v>21.23</v>
+      </c>
+      <c r="D98" s="2" t="n">
+        <v>21.23</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -4076,15 +3689,11 @@
           <t>1,500</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>26,94</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>40,41</t>
-        </is>
+      <c r="C99" s="2" t="n">
+        <v>26.94</v>
+      </c>
+      <c r="D99" s="2" t="n">
+        <v>40.41</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -4113,15 +3722,11 @@
           <t>1,500</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>26,94</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>40,41</t>
-        </is>
+      <c r="C100" s="2" t="n">
+        <v>26.94</v>
+      </c>
+      <c r="D100" s="2" t="n">
+        <v>40.41</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -4150,15 +3755,11 @@
           <t>1,500</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>26,94</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>40,41</t>
-        </is>
+      <c r="C101" s="2" t="n">
+        <v>26.94</v>
+      </c>
+      <c r="D101" s="2" t="n">
+        <v>40.41</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -4187,15 +3788,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>15,08</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>15,08</t>
-        </is>
+      <c r="C102" s="2" t="n">
+        <v>15.08</v>
+      </c>
+      <c r="D102" s="2" t="n">
+        <v>15.08</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -4224,15 +3821,11 @@
           <t>4,500</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>26,94</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>121,23</t>
-        </is>
+      <c r="C103" s="2" t="n">
+        <v>26.94</v>
+      </c>
+      <c r="D103" s="2" t="n">
+        <v>121.23</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -4261,15 +3854,11 @@
           <t>5,900</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>6,99</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>41,24</t>
-        </is>
+      <c r="C104" s="2" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="D104" s="2" t="n">
+        <v>41.24</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -4298,15 +3887,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>55,26</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>55,26</t>
-        </is>
+      <c r="C105" s="2" t="n">
+        <v>55.26</v>
+      </c>
+      <c r="D105" s="2" t="n">
+        <v>55.26</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -4335,15 +3920,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>30,47</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>30,47</t>
-        </is>
+      <c r="C106" s="2" t="n">
+        <v>30.47</v>
+      </c>
+      <c r="D106" s="2" t="n">
+        <v>30.47</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -4372,15 +3953,11 @@
           <t>1,000</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>18,19</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>18,19</t>
-        </is>
+      <c r="C107" s="2" t="n">
+        <v>18.19</v>
+      </c>
+      <c r="D107" s="2" t="n">
+        <v>18.19</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -4398,6 +3975,7 @@
         </is>
       </c>
     </row>
+    <row r="108"/>
     <row r="109">
       <c r="A109" t="inlineStr"/>
       <c r="B109" t="inlineStr"/>

</xml_diff>